<commit_message>
Document choice-bloc domain model and land year-3 curriculum research
CONTEXT.md: add Choice bloc, Curriculum option, Student choice, Teaching section, Choice vector; generalize Group partition/combination off single-Alternative.

docs/domain-model.md: clarify Alternative as one scalar implementation axis; record multi-bloc limitation with link to year-3 research.

docs/wayfinder/group-structure-2026-2027.md: blocs are audience-choice dimensions, not parallel-timeslot constraints; teaching-section terminology; sem-VI B4 numbering correction.

docs/wayfinder/year3-curriculum-website-research.md: official 2024 IA/I plan verification (6xo.1.1).

docs/wayfinder/inputs/2026-2027/: anonymized contingent + optional-course workbooks referenced by the grilling.

src/Features/Integration/data/2025_sem2/fr/2.xlsx: 326/6->326/4 room fix (2 cells).

Generated-by: Muse Spark (opencode/muse-spark)

Generated-by: Codex
</commit_message>
<xml_diff>
--- a/src/Features/Integration/data/2025_sem2/fr/2.xlsx
+++ b/src/Features/Integration/data/2025_sem2/fr/2.xlsx
@@ -2415,11 +2415,11 @@
       <c r="K34" s="13"/>
       <c r="L34" s="14" t="str">
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE""")," I: Design soft. (lab), 
-G-C. Stănescu, 326/6
+G-C. Stănescu, 326/4
  II: Cloud comp. (lab), 
 A. Prepeliță, 251/4")</f>
         <v xml:space="preserve"> I: Design soft. (lab), 
-G-C. Stănescu, 326/6
+G-C. Stănescu, 326/4
  II: Cloud comp. (lab), 
 A. Prepeliță, 251/4</v>
       </c>

</xml_diff>